<commit_message>
udpated project tracker and created docs
</commit_message>
<xml_diff>
--- a/data/project_tracker.xlsx
+++ b/data/project_tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81241728\Documents\PythonProjects\automation-project-tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13111F65-B3AE-4290-8A89-EF45112DD060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843F322B-B792-478F-B660-7B25CB27CDE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2740" yWindow="-14510" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="49">
   <si>
     <t>No</t>
   </si>
@@ -180,6 +180,9 @@
   </si>
   <si>
     <t>KCC</t>
+  </si>
+  <si>
+    <t>PepsiCo Browser SDK</t>
   </si>
 </sst>
 </file>
@@ -517,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="6.5234375" customWidth="1"/>
@@ -1237,11 +1240,63 @@
         <v>0</v>
       </c>
       <c r="N14" s="2">
-        <f t="shared" ref="N14" si="4">L14-M14</f>
+        <f t="shared" ref="N14:N15" si="4">L14-M14</f>
         <v>13</v>
       </c>
       <c r="O14" s="3">
-        <f t="shared" ref="O14" si="5">N14/L14</f>
+        <f t="shared" ref="O14:O15" si="5">N14/L14</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15">
+        <v>45</v>
+      </c>
+      <c r="I15">
+        <f>260*3</f>
+        <v>780</v>
+      </c>
+      <c r="J15">
+        <v>5</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2">
+        <f>(I15*J15)/60</f>
+        <v>65</v>
+      </c>
+      <c r="M15" s="2">
+        <f>(I15*K15)/60</f>
+        <v>0</v>
+      </c>
+      <c r="N15" s="2">
+        <f t="shared" si="4"/>
+        <v>65</v>
+      </c>
+      <c r="O15" s="3">
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated project tracker data
</commit_message>
<xml_diff>
--- a/data/project_tracker.xlsx
+++ b/data/project_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81241728\Documents\PythonProjects\automation-project-tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843F322B-B792-478F-B660-7B25CB27CDE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{623BCC41-F773-40F9-8316-46C5126A2B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2740" yWindow="-14510" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="50">
   <si>
     <t>No</t>
   </si>
@@ -183,6 +183,9 @@
   </si>
   <si>
     <t>PepsiCo Browser SDK</t>
+  </si>
+  <si>
+    <t>Perfect Store EDF uploads</t>
   </si>
 </sst>
 </file>
@@ -520,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="6.5234375" customWidth="1"/>
@@ -617,7 +620,7 @@
         <v>60</v>
       </c>
       <c r="K2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L2" s="2">
         <f>(I2*J2)/60</f>
@@ -625,15 +628,15 @@
       </c>
       <c r="M2" s="2">
         <f>(I2*K2)/60</f>
-        <v>43.333333333333336</v>
+        <v>21.666666666666668</v>
       </c>
       <c r="N2" s="2">
         <f>L2-M2</f>
-        <v>216.66666666666666</v>
+        <v>238.33333333333334</v>
       </c>
       <c r="O2" s="3">
         <f>N2/L2</f>
-        <v>0.83333333333333326</v>
+        <v>0.91666666666666674</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.55000000000000004">
@@ -668,7 +671,7 @@
         <v>120</v>
       </c>
       <c r="K3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L3" s="2">
         <f>(I3*J3)/60</f>
@@ -676,15 +679,15 @@
       </c>
       <c r="M3" s="2">
         <f t="shared" ref="M3:M12" si="0">(I3*K3)/60</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N3" s="2">
         <f t="shared" ref="N3:N13" si="1">L3-M3</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O3" s="3">
         <f t="shared" ref="O3:O13" si="2">N3/L3</f>
-        <v>0.91666666666666663</v>
+        <v>0.95833333333333337</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.55000000000000004">
@@ -1298,6 +1301,57 @@
       <c r="O15" s="3">
         <f t="shared" si="5"/>
         <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16">
+        <v>40</v>
+      </c>
+      <c r="I16">
+        <v>38</v>
+      </c>
+      <c r="J16">
+        <v>26</v>
+      </c>
+      <c r="K16">
+        <v>10</v>
+      </c>
+      <c r="L16" s="2">
+        <f>(I16*J16)/60</f>
+        <v>16.466666666666665</v>
+      </c>
+      <c r="M16" s="2">
+        <f>(I16*K16)/60</f>
+        <v>6.333333333333333</v>
+      </c>
+      <c r="N16" s="2">
+        <f t="shared" ref="N16" si="6">L16-M16</f>
+        <v>10.133333333333333</v>
+      </c>
+      <c r="O16" s="3">
+        <f t="shared" ref="O16" si="7">N16/L16</f>
+        <v>0.61538461538461542</v>
       </c>
     </row>
   </sheetData>

</xml_diff>